<commit_message>
fix(qa): align all remaining subspace QA.xlsx to official Wesome AI 3-column format
</commit_message>
<xml_diff>
--- a/subspaces/01-academic-training/academic-advisor-agent/agent/QA.xlsx
+++ b/subspaces/01-academic-training/academic-advisor-agent/agent/QA.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3597,7 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3618,7 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Không</t>
         </is>
       </c>
     </row>

</xml_diff>